<commit_message>
Final commit before April 28th presentation
</commit_message>
<xml_diff>
--- a/frontend/public/Red_Duke_Report.xlsx
+++ b/frontend/public/Red_Duke_Report.xlsx
@@ -53,22 +53,22 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00FFEBEE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00FFF3E0"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E8F5E9"/>
+        <fgColor rgb="00FF6630"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFEBEE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FF6630"/>
+        <fgColor rgb="00E8F5E9"/>
       </patternFill>
     </fill>
     <fill>
@@ -103,7 +103,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -119,19 +119,16 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -526,7 +523,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>ABC Corporation</t>
+          <t>DEF Insurance</t>
         </is>
       </c>
     </row>
@@ -538,7 +535,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>TG0 (Design)</t>
+          <t>TG-1 (Initiation)</t>
         </is>
       </c>
     </row>
@@ -562,7 +559,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>TG0 (Design)</t>
+          <t>TG-1 (Initiation)</t>
         </is>
       </c>
     </row>
@@ -578,7 +575,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>42%</t>
+          <t>10%</t>
         </is>
       </c>
     </row>
@@ -590,7 +587,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -602,7 +599,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -614,7 +611,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>22</t>
         </is>
       </c>
     </row>
@@ -626,7 +623,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>12</t>
         </is>
       </c>
     </row>
@@ -642,7 +639,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>1%</t>
+          <t>20%</t>
         </is>
       </c>
     </row>
@@ -706,7 +703,7 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>The ABC Corporation Virtual Mailroom project is currently in the Design (TG0) phase, with significant gaps in foundational documentation. The BRD is an early draft (v0.1) with critical placeholders, and key design documents like the Technical Design Specification and Data Mapping are missing. High-priority risks include the lack of defined client responsibilities and incomplete workflow specifications. To advance, the immediate focus must be on finalizing the BRD, completing core design documents, and defining reporting requirements and SLAs. Without these, proceeding to implementation and testing will be blocked.</t>
+          <t>The project is currently in a RED state due to significant gaps in foundational documentation, particularly the Business Requirements Document (BRD) and security documentation. Immediate action is required to complete these documents to align with project goals and timelines. The next steps involve scheduling a client kickoff meeting and developing essential documentation to facilitate progress.</t>
         </is>
       </c>
     </row>
@@ -730,7 +727,7 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>CONDITIONAL | Confidence: 45% | Risk: ? | Delay: 2-4 weeks</t>
+          <t>NO-GO | Confidence: 87% | Risk: ? | Delay: 1-2 months</t>
         </is>
       </c>
     </row>
@@ -742,7 +739,7 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>NO-GO | Confidence: 74% | Risk: ? | Delay: 3-6 weeks</t>
+          <t>NO-GO | Confidence: 100% | Risk: ? | Delay: 1-2 months</t>
         </is>
       </c>
     </row>
@@ -754,7 +751,7 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>NO-GO | Confidence: 81% | Risk: ? | Delay: 1-2 months</t>
+          <t>NO-GO | Confidence: 100% | Risk: ? | Delay: 1-2 months</t>
         </is>
       </c>
     </row>
@@ -766,7 +763,7 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>NO-GO | Confidence: 85% | Risk: ? | Delay: 1-2 months</t>
+          <t>NO-GO | Confidence: 100% | Risk: ? | Delay: 1-2 months</t>
         </is>
       </c>
     </row>
@@ -802,7 +799,7 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="19" customWidth="1" min="7" max="7"/>
     <col width="52" customWidth="1" min="8" max="8"/>
     <col width="52" customWidth="1" min="9" max="9"/>
   </cols>
@@ -872,12 +869,12 @@
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>PARTIAL</t>
+          <t>MISSING</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
@@ -887,17 +884,13 @@
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>Large</t>
-        </is>
-      </c>
-      <c r="H2" s="3" t="inlineStr">
-        <is>
-          <t>ABC Corporation 25080 BRD v0.1.docx</t>
-        </is>
-      </c>
+          <t>Large (3+ days)</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr"/>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>The BRD v0.1 exists but is incomplete, containing placeholders for critical client responsibilities and lacking details on reporting requirements and SLAs. It serves as a foundation but requires significant updates and sign-off.</t>
+          <t>The BRD is largely empty and lacks defined business requirements. It needs to be completed to move forward.</t>
         </is>
       </c>
     </row>
@@ -919,32 +912,32 @@
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
-          <t>PRESENT</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>MEDIUM</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>Small</t>
+          <t>Medium (1-3 days)</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>ABC Corporation - High-Level Critical Path Project Plan.docx</t>
+          <t>MY_Insurance_-_High-Level_Critical_Path_Project_Plan.docx</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>A detailed project plan outlining phases, timelines, and key activities is provided. It includes estimated durations and highlights overlapping tasks, serving as a clear roadmap for the project.</t>
+          <t>The project plan outlines the timeline but lacks detailed task descriptions. It needs to be expanded to provide clarity.</t>
         </is>
       </c>
     </row>
@@ -964,7 +957,7 @@
           <t>PM</t>
         </is>
       </c>
-      <c r="D4" s="7" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
@@ -976,18 +969,18 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Medium (1-3 days)</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr"/>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>While the project plan implies initiation activities like SOW sign-off and discovery sessions, there is no explicit documentation or mention of a formal client kickoff meeting or scope presentation within the provided documents.</t>
+          <t>No evidence of a kickoff meeting or scope presentation has been documented. This is essential for stakeholder alignment.</t>
         </is>
       </c>
     </row>
@@ -1009,32 +1002,28 @@
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>PARTIAL</t>
+          <t>MISSING</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="H5" s="3" t="inlineStr">
-        <is>
-          <t>ABC Corporation 25080 BRD v0.1.docx</t>
-        </is>
-      </c>
+          <t>Large (3+ days)</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr"/>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>The BRD mentions SFTP connectivity details including URL, username, port, and SSH key, and IP whitelisting. However, comprehensive security and access control documentation beyond these SFTP specifics is not evident.</t>
+          <t>No documentation regarding security and access controls has been provided. This is critical for compliance.</t>
         </is>
       </c>
     </row>
@@ -1054,7 +1043,7 @@
           <t>PM</t>
         </is>
       </c>
-      <c r="D6" s="7" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
@@ -1066,18 +1055,18 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>Large</t>
+          <t>Medium (1-3 days)</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr"/>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>There is no mention or evidence of training materials or process awareness documentation within the provided files. This is a critical deliverable for client adoption and operational handover.</t>
+          <t>No training materials or process awareness documentation has been created. This is necessary for user adoption.</t>
         </is>
       </c>
     </row>
@@ -1099,12 +1088,12 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>PARTIAL</t>
+          <t>MISSING</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
@@ -1114,17 +1103,13 @@
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="H7" s="3" t="inlineStr">
-        <is>
-          <t>ABC Corporation -WF Diagram.vsdx</t>
-        </is>
-      </c>
+          <t>Large (3+ days)</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr"/>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>Multiple workflow diagrams are provided, illustrating various aspects of the process. However, the diagrams are explicitly marked as 'illustrative' and not the definitive 'Proposed Solution', indicating they are a starting point but not a final design.</t>
+          <t>No workflow diagrams have been created. This is essential for visualizing the process.</t>
         </is>
       </c>
     </row>
@@ -1144,7 +1129,7 @@
           <t>Engineering</t>
         </is>
       </c>
-      <c r="D8" s="7" t="inlineStr">
+      <c r="D8" s="5" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
@@ -1161,13 +1146,13 @@
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>Large</t>
+          <t>Large (3+ days)</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr"/>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>No data mapping document is present. While the BRD mentions input/output file specifications and the project plan lists 'Sync-up on Input and Output file specifications', the actual mapping details are missing.</t>
+          <t>No data mapping documentation has been provided. This is critical for ensuring data flows correctly.</t>
         </is>
       </c>
     </row>
@@ -1187,10 +1172,14 @@
           <t>Engineering</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr"/>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>MISSING</t>
+        </is>
+      </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
@@ -1200,17 +1189,13 @@
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>Large</t>
-        </is>
-      </c>
-      <c r="H9" s="3" t="inlineStr">
-        <is>
-          <t>ABC Corporation -WF Diagram.vsdx, ABC Corporation 25080 BRD v0.1.docx</t>
-        </is>
-      </c>
+          <t>Large (3+ days)</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr"/>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>The BRD provides some technical details for SFTP connectivity and client-performed scanning integration. The WF Diagram offers a high-level process flow. However, a comprehensive Technical Design Specification detailing system architecture, integrations, and specific configurations is not present.</t>
+          <t>No technical design specifications have been documented. This is necessary for guiding development.</t>
         </is>
       </c>
     </row>
@@ -1230,7 +1215,7 @@
           <t>Business Analyst / PM</t>
         </is>
       </c>
-      <c r="D10" s="7" t="inlineStr">
+      <c r="D10" s="5" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
@@ -1247,13 +1232,13 @@
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>Small</t>
+          <t>Medium (1-3 days)</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr"/>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>The BRD is version v0.1 and contains placeholders, indicating it is not finalized. There is no evidence of client sign-off on the BRD.</t>
+          <t>No sign-off on the BRD has been documented. This is essential for moving forward.</t>
         </is>
       </c>
     </row>
@@ -1273,7 +1258,7 @@
           <t>PM / Engineering</t>
         </is>
       </c>
-      <c r="D11" s="7" t="inlineStr">
+      <c r="D11" s="5" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
@@ -1285,18 +1270,18 @@
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>Large</t>
+          <t>Medium (1-3 days)</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr"/>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>No implementation or transition workbook is mentioned or provided. This is a key document for detailing the steps and responsibilities for moving from design to production.</t>
+          <t>No implementation workbook has been created. This is necessary for tracking implementation tasks.</t>
         </is>
       </c>
     </row>
@@ -1316,10 +1301,14 @@
           <t>Engineering</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr"/>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>MISSING</t>
+        </is>
+      </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
@@ -1329,17 +1318,13 @@
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>Large</t>
-        </is>
-      </c>
-      <c r="H12" s="3" t="inlineStr">
-        <is>
-          <t>ABC Corporation 25080 BRD v0.1.docx</t>
-        </is>
-      </c>
+          <t>Large (3+ days)</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr"/>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>The BRD provides some configuration details for SFTP connectivity and intake folder structures. However, comprehensive configuration documentation for mailroom, workflow, and other system settings is not present.</t>
+          <t>No configuration documentation has been provided. This is critical for system setup.</t>
         </is>
       </c>
     </row>
@@ -1359,7 +1344,7 @@
           <t>PM</t>
         </is>
       </c>
-      <c r="D13" s="7" t="inlineStr">
+      <c r="D13" s="5" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
@@ -1371,18 +1356,18 @@
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Medium (1-3 days)</t>
         </is>
       </c>
       <c r="H13" s="3" t="inlineStr"/>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>The Project Plan mentions 'Client access, Reporting Requirement and SLA' as a task, but no specific documentation detailing these requirements or SLAs is provided.</t>
+          <t>No reporting requirements or SLA documentation has been created. This is necessary for performance tracking.</t>
         </is>
       </c>
     </row>
@@ -1402,10 +1387,14 @@
           <t>Engineering</t>
         </is>
       </c>
-      <c r="D14" s="3" t="inlineStr"/>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>MISSING</t>
+        </is>
+      </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
@@ -1415,17 +1404,13 @@
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>Large</t>
-        </is>
-      </c>
-      <c r="H14" s="3" t="inlineStr">
-        <is>
-          <t>ABC Corporation -WF Diagram.vsdx, ABC Corporation 25080 BRD v0.1.docx</t>
-        </is>
-      </c>
+          <t>Large (3+ days)</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr"/>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>The WF Diagram provides a high-level overview of the workflow, and the BRD outlines intake channels and SFTP structure. However, detailed configuration specifications for the mailroom and specific workflow rules are not present.</t>
+          <t>No mailroom configuration documentation has been provided. This is critical for system functionality.</t>
         </is>
       </c>
     </row>
@@ -1445,10 +1430,14 @@
           <t>Engineering</t>
         </is>
       </c>
-      <c r="D15" s="3" t="inlineStr"/>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>MISSING</t>
+        </is>
+      </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
@@ -1458,17 +1447,13 @@
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>Large</t>
-        </is>
-      </c>
-      <c r="H15" s="3" t="inlineStr">
-        <is>
-          <t>ABC Corporation 25080 BRD v0.1.docx</t>
-        </is>
-      </c>
+          <t>Large (3+ days)</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr"/>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>The BRD mentions 'Eligibility Matching' in the context of workflow and lists 'Sample Files: One week’s worth of each document type (e.g., claims, EOBs, correspondence)' and 'Eligibility &amp; Provider Files: Current format/layout and sample data' as critical early deliverables. However, specific configuration details for eligibility and claims processing are not provided.</t>
+          <t>No eligibility and claims configuration documentation has been provided. This is necessary for claims processing.</t>
         </is>
       </c>
     </row>
@@ -1488,10 +1473,14 @@
           <t>Engineering / PM</t>
         </is>
       </c>
-      <c r="D16" s="3" t="inlineStr"/>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>MISSING</t>
+        </is>
+      </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
@@ -1501,17 +1490,13 @@
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>Large</t>
-        </is>
-      </c>
-      <c r="H16" s="3" t="inlineStr">
-        <is>
-          <t>ABC Corporation - High-Level Critical Path Project Plan.docx</t>
-        </is>
-      </c>
+          <t>Large (3+ days)</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="inlineStr"/>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>The Project Plan mentions 'Preparing test cases and samples' (10 days) and 'UAT by client' (10 days) within the Testing phase. However, a formal UAT Plan and specific test cases are not provided.</t>
+          <t>No UAT plan or test cases have been documented. This is essential for validating the implementation.</t>
         </is>
       </c>
     </row>
@@ -1531,7 +1516,7 @@
           <t>Engineering</t>
         </is>
       </c>
-      <c r="D17" s="7" t="inlineStr">
+      <c r="D17" s="5" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
@@ -1548,13 +1533,13 @@
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Large (3+ days)</t>
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr"/>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>As UAT is planned but no plan or test cases exist, there is no evidence of UAT sign-off or testing evidence.</t>
+          <t>No UAT sign-off or testing evidence has been documented. This is critical for project validation.</t>
         </is>
       </c>
     </row>
@@ -1574,7 +1559,7 @@
           <t>PM / Engineer</t>
         </is>
       </c>
-      <c r="D18" s="7" t="inlineStr">
+      <c r="D18" s="5" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
@@ -1586,18 +1571,18 @@
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Medium (1-3 days)</t>
         </is>
       </c>
       <c r="H18" s="3" t="inlineStr"/>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>There is no mention or evidence of a TPM or compliance checklist within the provided documents.</t>
+          <t>No compliance checklist has been created. This is necessary for ensuring regulatory adherence.</t>
         </is>
       </c>
     </row>
@@ -1617,10 +1602,14 @@
           <t>Engineering</t>
         </is>
       </c>
-      <c r="D19" s="3" t="inlineStr"/>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>MISSING</t>
+        </is>
+      </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
@@ -1630,17 +1619,13 @@
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="H19" s="3" t="inlineStr">
-        <is>
-          <t>ABC Corporation - High-Level Critical Path Project Plan.docx</t>
-        </is>
-      </c>
+          <t>Large (3+ days)</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr"/>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>The Project Plan lists 'Functional testing of non-claims' and 'Volume testing' as activities. However, no specific evidence or documentation of these tests having been performed or their results is provided.</t>
+          <t>No functional or volume testing evidence has been documented. This is critical for validating system performance.</t>
         </is>
       </c>
     </row>
@@ -1660,7 +1645,7 @@
           <t>PM / Tech Lead</t>
         </is>
       </c>
-      <c r="D20" s="7" t="inlineStr">
+      <c r="D20" s="5" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
@@ -1677,13 +1662,13 @@
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>Small</t>
+          <t>Medium (1-3 days)</t>
         </is>
       </c>
       <c r="H20" s="3" t="inlineStr"/>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>As the project appears to be in the Design phase with many implementation and testing deliverables missing, there is no evidence of a Go-Live sign-off.</t>
+          <t>No Go-Live sign-off has been documented. This is essential for project closure.</t>
         </is>
       </c>
     </row>
@@ -1703,7 +1688,7 @@
           <t>PM</t>
         </is>
       </c>
-      <c r="D21" s="7" t="inlineStr">
+      <c r="D21" s="5" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
@@ -1720,13 +1705,13 @@
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>Small</t>
+          <t>Medium (1-3 days)</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr"/>
       <c r="I21" s="3" t="inlineStr">
         <is>
-          <t>No documentation related to post-go-live warranty or checklists is available.</t>
+          <t>No post-Go-Live warranty checklist has been created. This is necessary for ensuring ongoing support.</t>
         </is>
       </c>
     </row>
@@ -1746,7 +1731,7 @@
           <t>PM</t>
         </is>
       </c>
-      <c r="D22" s="7" t="inlineStr">
+      <c r="D22" s="5" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
@@ -1763,13 +1748,13 @@
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>Small</t>
+          <t>Medium (1-3 days)</t>
         </is>
       </c>
       <c r="H22" s="3" t="inlineStr"/>
       <c r="I22" s="3" t="inlineStr">
         <is>
-          <t>This deliverable is for post-deployment. As the project is in the design phase, no lessons learned document would exist yet.</t>
+          <t>No lessons learned document has been created. This is important for future projects.</t>
         </is>
       </c>
     </row>
@@ -1789,7 +1774,7 @@
           <t>PM</t>
         </is>
       </c>
-      <c r="D23" s="7" t="inlineStr">
+      <c r="D23" s="5" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
@@ -1801,18 +1786,18 @@
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Medium (1-3 days)</t>
         </is>
       </c>
       <c r="H23" s="3" t="inlineStr"/>
       <c r="I23" s="3" t="inlineStr">
         <is>
-          <t>This is a final deliverable. Given the project's current stage and numerous missing items, this is not yet available.</t>
+          <t>No final documentation handoff has been documented. This is critical for project closure.</t>
         </is>
       </c>
     </row>
@@ -1827,50 +1812,50 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="23" customWidth="1" min="3" max="3"/>
     <col width="52" customWidth="1" min="4" max="4"/>
-    <col width="19" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="46" customWidth="1" min="7" max="7"/>
+    <col width="23" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="8" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>Gap</t>
         </is>
       </c>
-      <c r="B1" s="8" t="inlineStr">
+      <c r="B1" s="7" t="inlineStr">
         <is>
           <t>Impact</t>
         </is>
       </c>
-      <c r="C1" s="8" t="inlineStr">
+      <c r="C1" s="7" t="inlineStr">
         <is>
           <t>Stage Gate</t>
         </is>
       </c>
-      <c r="D1" s="8" t="inlineStr">
+      <c r="D1" s="7" t="inlineStr">
         <is>
           <t>Recommendation</t>
         </is>
       </c>
-      <c r="E1" s="8" t="inlineStr">
+      <c r="E1" s="7" t="inlineStr">
         <is>
           <t>Responsible Party</t>
         </is>
       </c>
-      <c r="F1" s="8" t="inlineStr">
+      <c r="F1" s="7" t="inlineStr">
         <is>
           <t>Est. Effort</t>
         </is>
       </c>
-      <c r="G1" s="8" t="inlineStr">
+      <c r="G1" s="7" t="inlineStr">
         <is>
           <t>Dependencies</t>
         </is>
@@ -1879,22 +1864,22 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>BRD v0.1 contains placeholders for critical client responsibilities regarding pre-scan document preparation and indexing (e.g., document separation, identification, sorting).</t>
-        </is>
-      </c>
-      <c r="B2" s="7" t="inlineStr">
+          <t>Business Requirements Document (BRD) is largely empty and lacks defined business requirements.</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>TG0 (Design)</t>
+          <t>TG-1 (Initiation)</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>Schedule a dedicated session with ABC Corporation SMEs to define and document these specific responsibilities within the BRD. Update the BRD with concrete details and obtain client sign-off.</t>
+          <t>Complete the BRD with detailed business requirements.</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
@@ -1904,7 +1889,7 @@
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Large (3+ days)</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr"/>
@@ -1912,59 +1897,55 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Lack of detailed Technical Design Specification, Data Mapping Document, and finalized Workflow/Process Flow Diagram.</t>
-        </is>
-      </c>
-      <c r="B3" s="7" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+          <t>High-Level Project Plan lacks detailed task descriptions.</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>TG0 (Design)</t>
+          <t>TG-1 (Initiation)</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Engineering team to develop a comprehensive Technical Design Specification, including detailed data mapping and finalize the workflow diagram based on the 'Proposed Solution' referenced in the Visio file. Obtain client review and sign-off.</t>
+          <t>Expand the project plan to include detailed tasks and deadlines.</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Engineering</t>
+          <t>PM</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Large</t>
-        </is>
-      </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>BRD Sign-off</t>
-        </is>
-      </c>
+          <t>Medium (1-3 days)</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Reporting Requirements &amp; SLA Documentation is missing.</t>
-        </is>
-      </c>
-      <c r="B4" s="7" t="inlineStr">
+          <t>No Client Kickoff / Scope Presentation has been documented.</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>TG1 (Implementation)</t>
+          <t>TG-1 (Initiation)</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Schedule a meeting with ABC Corporation to define and document all reporting requirements and Service Level Agreements (SLAs). Create a formal document for client review and sign-off.</t>
+          <t>Schedule and document a client kickoff meeting.</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -1974,71 +1955,63 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>BRD Sign-off</t>
-        </is>
-      </c>
+          <t>Medium (1-3 days)</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Absence of formal UAT Plan &amp; Test Cases.</t>
-        </is>
-      </c>
-      <c r="B5" s="7" t="inlineStr">
+          <t>No Security &amp; Access Control Documentation has been provided.</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>TG2 (Test)</t>
+          <t>TG-1 (Initiation)</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Develop a comprehensive UAT Plan and detailed test cases based on the finalized requirements and technical design. Engage ABC Corporation for review and approval.</t>
+          <t>Create security and access control documentation.</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>Engineering / PM</t>
+          <t>Engineering</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Large</t>
-        </is>
-      </c>
-      <c r="G5" s="3" t="inlineStr">
-        <is>
-          <t>Technical Design Specification, BRD Sign-off</t>
-        </is>
-      </c>
+          <t>Large (3+ days)</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>No evidence of Training &amp; Process Awareness Documentation.</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
+          <t>No Training &amp; Process Awareness Documentation has been created.</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>TG1 (Implementation)</t>
+          <t>TG-1 (Initiation)</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Develop training materials and process documentation for ABC Corporation end-users and support staff. This should cover system usage, workflows, and support procedures.</t>
+          <t>Develop training materials for user adoption.</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
@@ -2048,34 +2021,30 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Large</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="inlineStr">
-        <is>
-          <t>Configuration Documentation</t>
-        </is>
-      </c>
+          <t>Medium (1-3 days)</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Security &amp; Access Control Documentation beyond SFTP specifics is not comprehensive.</t>
+          <t>No Workflow / Process Flow Diagram has been created.</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>TG1 (Implementation)</t>
+          <t>TG0 (Design)</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Expand on the existing SFTP security details to include broader access control policies, user roles, and data security measures relevant to the SDS platform.</t>
+          <t>Create a workflow/process flow diagram.</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -2085,7 +2054,7 @@
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Large (3+ days)</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr"/>
@@ -2093,35 +2062,530 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>No formal Client Kickoff / Scope Presentation documented.</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
+          <t>No Data Mapping Document has been provided.</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>TG0 (Design)</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Develop a data mapping document.</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Large (3+ days)</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>No Technical Design Specification has been documented.</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>TG0 (Design)</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Create a technical design specification.</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>Large (3+ days)</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>No BRD Sign-off has been documented.</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>TG0 (Design)</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Obtain sign-off on the BRD.</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Business Analyst / PM</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>Medium (1-3 days)</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>No Implementation / Transition Workbook has been created.</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>TG1 (Implementation)</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Develop an implementation workbook.</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>PM / Engineering</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Medium (1-3 days)</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>No Configuration Documentation has been provided.</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>TG1 (Implementation)</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Create configuration documentation.</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>Large (3+ days)</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>No Reporting Requirements &amp; SLA Documentation has been created.</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>TG1 (Implementation)</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Develop reporting requirements and SLA documentation.</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>Medium (1-3 days)</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>No Mailroom / Workflow Configuration documentation has been provided.</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>TG1 (Implementation)</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>Create mailroom/workflow configuration documentation.</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>Large (3+ days)</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>No Eligibility &amp; Claims Configuration documentation has been provided.</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>TG1 (Implementation)</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Develop eligibility and claims configuration documentation.</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>Large (3+ days)</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>No UAT Plan &amp; Test Cases have been documented.</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>TG2 (Test)</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>Create a UAT plan and test cases.</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>Engineering / PM</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>Large (3+ days)</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>No UAT Sign-off / Testing Evidence has been documented.</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>TG2 (Test)</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Obtain UAT sign-off and document testing evidence.</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>Large (3+ days)</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>No TPM / Compliance Checklist has been created.</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>TG2 (Test)</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>Develop a TPM/compliance checklist.</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>PM / Engineer</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>Medium (1-3 days)</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>No Functional &amp; Volume Testing Evidence has been documented.</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>TG2 (Test)</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>Document functional and volume testing evidence.</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>Large (3+ days)</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>No M2P / Go-Live Sign-off has been documented.</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>TG3 (Deploy/Warranty)</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>Obtain Go-Live sign-off.</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>PM / Tech Lead</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>Medium (1-3 days)</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>No Post-Go-Live Warranty Checklist has been created.</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>TG3 (Deploy/Warranty)</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>Develop a post-Go-Live warranty checklist.</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>Medium (1-3 days)</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>No Lessons Learned Document has been created.</t>
+        </is>
+      </c>
+      <c r="B22" s="8" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>TG-1 (Initiation)</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>Confirm if a client kickoff meeting occurred. If not, schedule one to formally align on scope, project plan, and expectations. Document the meeting outcomes.</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>TG3 (Deploy/Warranty)</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>Create a lessons learned document.</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
         <is>
           <t>PM</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>Small</t>
-        </is>
-      </c>
-      <c r="G8" s="3" t="inlineStr"/>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>Medium (1-3 days)</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>No Final Client Documentation Handoff has been documented.</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>TG3 (Deploy/Warranty)</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>Document the final client documentation handoff.</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>Medium (1-3 days)</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2134,16 +2598,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="52" customWidth="1" min="2" max="2"/>
     <col width="23" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="23" customWidth="1" min="5" max="5"/>
     <col width="44" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="19" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2189,7 +2653,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Schedule and conduct a session with ABC Corporation SMEs to define and document pre-scan preparation and indexing responsibilities in the BRD.</t>
+          <t>Complete the Business Requirements Document (BRD) with detailed business requirements.</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
@@ -2204,7 +2668,7 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>TG0 (Design)</t>
+          <t>TG-1 (Initiation)</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
@@ -2214,7 +2678,7 @@
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Large (3+ days)</t>
         </is>
       </c>
     </row>
@@ -2224,32 +2688,32 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Develop a comprehensive Technical Design Specification, including detailed data mapping and finalize the workflow diagram based on the 'Proposed Solution'.</t>
+          <t>Expand the High-Level Project Plan to include detailed tasks and deadlines.</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Engineering</t>
+          <t>PM</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>TG0 (Design)</t>
+          <t>TG-1 (Initiation)</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Technical Design Specification</t>
+          <t>High-Level Project Plan / Critical Path</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>Large</t>
+          <t>Medium (1-3 days)</t>
         </is>
       </c>
     </row>
@@ -2259,7 +2723,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Define and document Reporting Requirements &amp; SLAs with ABC Corporation.</t>
+          <t>Schedule and document a client kickoff meeting.</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -2274,17 +2738,17 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>TG1 (Implementation)</t>
+          <t>TG-1 (Initiation)</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Reporting Requirements &amp; SLA Documentation</t>
+          <t>Client Kickoff / Scope Presentation</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Medium (1-3 days)</t>
         </is>
       </c>
     </row>
@@ -2294,12 +2758,12 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Develop a formal UAT Plan and detailed test cases.</t>
+          <t>Create security and access control documentation.</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Engineering / PM</t>
+          <t>Engineering</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -2309,17 +2773,17 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>TG2 (Test)</t>
+          <t>TG-1 (Initiation)</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>UAT Plan &amp; Test Cases</t>
+          <t>Security &amp; Access Control Documentation</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>Large</t>
+          <t>Large (3+ days)</t>
         </is>
       </c>
     </row>
@@ -2329,32 +2793,32 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Obtain client sign-off on the updated BRD.</t>
+          <t>Develop training materials for user adoption.</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Business Analyst / PM</t>
+          <t>PM</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>TG0 (Design)</t>
+          <t>TG-1 (Initiation)</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>BRD Sign-off</t>
+          <t>Training &amp; Process Awareness Documentation</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>Small</t>
+          <t>Medium (1-3 days)</t>
         </is>
       </c>
     </row>
@@ -2364,12 +2828,12 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Develop Training &amp; Process Awareness Documentation.</t>
+          <t>Create a workflow/process flow diagram.</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>PM</t>
+          <t>Engineering</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -2379,17 +2843,17 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>TG1 (Implementation)</t>
+          <t>TG0 (Design)</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Training &amp; Process Awareness Documentation</t>
+          <t>Workflow / Process Flow Diagram</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>Large</t>
+          <t>Large (3+ days)</t>
         </is>
       </c>
     </row>
@@ -2399,7 +2863,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Finalize and document comprehensive Security &amp; Access Control measures.</t>
+          <t>Develop a data mapping document.</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -2409,22 +2873,22 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>TG1 (Implementation)</t>
+          <t>TG0 (Design)</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>Security &amp; Access Control Documentation</t>
+          <t>Data Mapping Document</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Large (3+ days)</t>
         </is>
       </c>
     </row>
@@ -2434,32 +2898,32 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Confirm occurrence of Client Kickoff / Scope Presentation and document outcomes if not already done.</t>
+          <t>Create a technical design specification.</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>PM</t>
+          <t>Engineering</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>TG-1 (Initiation)</t>
+          <t>TG0 (Design)</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>Client Kickoff / Scope Presentation</t>
+          <t>Technical Design Specification</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>Small</t>
+          <t>Large (3+ days)</t>
         </is>
       </c>
     </row>
@@ -2469,12 +2933,12 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Develop Implementation / Transition Workbook.</t>
+          <t>Obtain sign-off on the BRD.</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>PM / Engineering</t>
+          <t>Business Analyst / PM</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
@@ -2484,17 +2948,17 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>TG1 (Implementation)</t>
+          <t>TG0 (Design)</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>Implementation / Transition Workbook</t>
+          <t>BRD Sign-off</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>Large</t>
+          <t>Medium (1-3 days)</t>
         </is>
       </c>
     </row>
@@ -2504,17 +2968,17 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Create comprehensive Configuration Documentation.</t>
+          <t>Develop an implementation workbook.</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Engineering</t>
+          <t>PM / Engineering</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
@@ -2524,12 +2988,12 @@
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Configuration Documentation</t>
+          <t>Implementation / Transition Workbook</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>Large</t>
+          <t>Medium (1-3 days)</t>
         </is>
       </c>
     </row>
@@ -2539,7 +3003,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Develop Mailroom / Workflow Configuration details.</t>
+          <t>Create configuration documentation.</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -2559,12 +3023,12 @@
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>Mailroom / Workflow Configuration</t>
+          <t>Configuration Documentation</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>Large</t>
+          <t>Large (3+ days)</t>
         </is>
       </c>
     </row>
@@ -2574,17 +3038,17 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Develop Eligibility &amp; Claims Configuration details.</t>
+          <t>Develop reporting requirements and SLA documentation.</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Engineering</t>
+          <t>PM</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
@@ -2594,12 +3058,12 @@
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>Eligibility &amp; Claims Configuration</t>
+          <t>Reporting Requirements &amp; SLA Documentation</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>Large</t>
+          <t>Medium (1-3 days)</t>
         </is>
       </c>
     </row>
@@ -2609,7 +3073,7 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Prepare Functional &amp; Volume Testing Evidence.</t>
+          <t>Create mailroom/workflow configuration documentation.</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
@@ -2624,17 +3088,332 @@
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
+          <t>TG1 (Implementation)</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>Mailroom / Workflow Configuration</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>Large (3+ days)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Develop eligibility and claims configuration documentation.</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>TG1 (Implementation)</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>Eligibility &amp; Claims Configuration</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>Large (3+ days)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Create a UAT plan and test cases.</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Engineering / PM</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
           <t>TG2 (Test)</t>
         </is>
       </c>
-      <c r="F14" s="3" t="inlineStr">
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>UAT Plan &amp; Test Cases</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>Large (3+ days)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Obtain UAT sign-off and document testing evidence.</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>TG2 (Test)</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>UAT Sign-off / Testing Evidence</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>Large (3+ days)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Develop a TPM/compliance checklist.</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>PM / Engineer</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>TG2 (Test)</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>TPM / Compliance Checklist</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>Medium (1-3 days)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Document functional and volume testing evidence.</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>TG2 (Test)</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
         <is>
           <t>Functional &amp; Volume Testing Evidence</t>
         </is>
       </c>
-      <c r="G14" s="3" t="inlineStr">
-        <is>
-          <t>Medium</t>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>Large (3+ days)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Obtain Go-Live sign-off.</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>PM / Tech Lead</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>TG3 (Deploy/Warranty)</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>M2P / Go-Live Sign-off</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>Medium (1-3 days)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Develop a post-Go-Live warranty checklist.</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>TG3 (Deploy/Warranty)</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>Post-Go-Live Warranty Checklist</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>Medium (1-3 days)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Create a lessons learned document.</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>TG3 (Deploy/Warranty)</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>Lessons Learned Document</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>Medium (1-3 days)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Document the final client documentation handoff.</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>TG3 (Deploy/Warranty)</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>Final Client Documentation Handoff</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>Medium (1-3 days)</t>
         </is>
       </c>
     </row>
@@ -2653,7 +3432,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
@@ -2724,43 +3503,43 @@
       </c>
       <c r="B2" s="10" t="inlineStr">
         <is>
-          <t>CONDITIONAL</t>
+          <t>NO-GO</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>45%</t>
+          <t>87%</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr"/>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>40%</t>
+          <t>10%</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>2-4 weeks</t>
+          <t>1-2 months</t>
         </is>
       </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
-          <t>Partial readiness at 45%. 4 blocker(s) remain: Business Requirements Document (BRD), Client Kickoff / Scope Presentation, Security &amp; Access Control Documentation. Gate passage is possible once these items are addressed.</t>
+          <t>Readiness score is 13% — well below the threshold. 4 deliverable(s) are MISSING: Business Requirements Document (BRD), Client Kickoff / Scope Presentation, Security &amp; Access Control Documentation. Significant work is needed before this gate can be considered.</t>
         </is>
       </c>
     </row>
@@ -2770,20 +3549,20 @@
           <t>TG0</t>
         </is>
       </c>
-      <c r="B3" s="11" t="inlineStr">
+      <c r="B3" s="10" t="inlineStr">
         <is>
           <t>NO-GO</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>74%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr"/>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>12%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
@@ -2803,12 +3582,12 @@
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>3-6 weeks</t>
+          <t>1-2 months</t>
         </is>
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>Readiness score is 26% — well below the threshold. 3 deliverable(s) are MISSING: Data Mapping Document, Technical Design Specification, BRD Sign-off. Significant work is needed before this gate can be considered.</t>
+          <t>Readiness score is 0% — well below the threshold. 4 deliverable(s) are MISSING: Workflow / Process Flow Diagram, Data Mapping Document, Technical Design Specification. Significant work is needed before this gate can be considered.</t>
         </is>
       </c>
     </row>
@@ -2818,14 +3597,14 @@
           <t>TG1</t>
         </is>
       </c>
-      <c r="B4" s="11" t="inlineStr">
+      <c r="B4" s="10" t="inlineStr">
         <is>
           <t>NO-GO</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>81%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr"/>
@@ -2856,7 +3635,7 @@
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>Readiness score is 19% — well below the threshold. 5 deliverable(s) are MISSING: Implementation / Transition Workbook, Configuration Documentation, Reporting Requirements &amp; SLA Documentation. Significant work is needed before this gate can be considered.</t>
+          <t>Readiness score is 0% — well below the threshold. 5 deliverable(s) are MISSING: Implementation / Transition Workbook, Configuration Documentation, Reporting Requirements &amp; SLA Documentation. Significant work is needed before this gate can be considered.</t>
         </is>
       </c>
     </row>
@@ -2866,14 +3645,14 @@
           <t>TG2</t>
         </is>
       </c>
-      <c r="B5" s="11" t="inlineStr">
+      <c r="B5" s="10" t="inlineStr">
         <is>
           <t>NO-GO</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>85%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr"/>
@@ -2904,7 +3683,7 @@
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>Readiness score is 15% — well below the threshold. 4 deliverable(s) are MISSING: UAT Plan &amp; Test Cases, UAT Sign-off / Testing Evidence, TPM / Compliance Checklist. Significant work is needed before this gate can be considered.</t>
+          <t>Readiness score is 0% — well below the threshold. 4 deliverable(s) are MISSING: UAT Plan &amp; Test Cases, UAT Sign-off / Testing Evidence, TPM / Compliance Checklist. Significant work is needed before this gate can be considered.</t>
         </is>
       </c>
     </row>
@@ -2914,7 +3693,7 @@
           <t>TG3</t>
         </is>
       </c>
-      <c r="B6" s="11" t="inlineStr">
+      <c r="B6" s="10" t="inlineStr">
         <is>
           <t>NO-GO</t>
         </is>
@@ -2942,7 +3721,7 @@
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I6" s="3" t="inlineStr">

</xml_diff>